<commit_message>
Actualiza diseño y archivos de la aplicación
</commit_message>
<xml_diff>
--- a/salidas/TIEMPOS_TAPA_PLASTICA_2026_MAY_DILIGENCIADO.xlsx
+++ b/salidas/TIEMPOS_TAPA_PLASTICA_2026_MAY_DILIGENCIADO.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diego\Desktop\CCM_MANTENIMIENTO\formatos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Diego\Desktop\CCM_MANTENIMIENTO\salidas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EF207C3-96B0-4CF3-A14F-9E074A2EAFD2}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{456936E0-718B-4FB4-95D9-523D6FA99AE1}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="637" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5115" yWindow="2925" windowWidth="15375" windowHeight="7875" tabRatio="637" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TPIBPHG11" sheetId="48" state="hidden" r:id="rId1"/>
@@ -91,8 +91,862 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Diego</author>
+  </authors>
+  <commentList>
+    <comment ref="H10" authorId="0" shapeId="0" xr:uid="{194CBC02-603C-4E23-9950-312857609936}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>fuga de agua</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C13" authorId="0" shapeId="0" xr:uid="{6D892E31-3D6C-4DD4-B1ED-CCC6EBAC2CDE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revision zonas boquilla y cuerpo casquilo se suben de temperatura por encima del set poin.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D13" authorId="0" shapeId="0" xr:uid="{BA9AC278-E98D-4AA2-832B-0FA5CAAB8B47}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>BLOQUEO POR ALARMA CONTROLADOR SP20</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F13" authorId="0" shapeId="0" xr:uid="{6B960B66-FBFF-4B10-B607-6318B558AC45}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>PERDIDA DE SINCRONISMO FSM</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H13" authorId="0" shapeId="0" xr:uid="{8E3CB650-C490-4AF8-A12B-8E3C61889B2B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revision daño de racor punzon #39 (fuga de agua)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C14" authorId="0" shapeId="0" xr:uid="{1EB526EC-E31D-45AA-B44F-0271B3BD1137}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Entortamiento carrusel de insercion.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D14" authorId="0" shapeId="0" xr:uid="{EABD8A9D-2588-4518-93ED-C80D7C392672}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>1. Parada por alarma SP18
+2. Bajar Encoder  Carrusel de Corte en la FSM 3
+3. Cambiar encoder carrusel en la FSM 3 Por que se paso para habilitar la FMS 5 CCM5
+4. Alarma SP20</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F14" authorId="0" shapeId="0" xr:uid="{65FC18FB-079C-4EED-82C8-5DD432F3A029}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>FALLA SINCRONISMO CARRUSELES</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C15" authorId="0" shapeId="0" xr:uid="{476CA739-948C-41C3-987C-93CEDD425CFA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Entortamiento carrusel de insercion.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D15" authorId="0" shapeId="0" xr:uid="{ABE1A36B-CBB5-4044-9D48-C0B16C5498C0}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>1. Alarma SP20
+2. alarma BQ8 encoder</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G15" authorId="0" shapeId="0" xr:uid="{795B54F5-E810-4111-9E3A-E224E1E3DBD5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>1. tapa con anillo doblado recalentamiento en punzon
+2. bloque de presion en tapa deformada refrigeracion en punzones defisiente</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B16" authorId="0" shapeId="0" xr:uid="{98C09E13-3F02-4688-9412-BAD805312AF4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revision calbibracion de cuchillas</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D16" authorId="0" shapeId="0" xr:uid="{8138630A-12A9-4209-8DAB-C0602D4BF7A7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>1. Temperatura alta en la zona de la bomba y fuga de agua cavidad 14.
+2. Temperatura alta en la zona de la bomba y fuga de ahua cavidad 14.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B17" authorId="0" shapeId="0" xr:uid="{13D56E6C-ADCB-410B-8C12-AD7DCD33DE62}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revision pantalla CVS - No prende</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G17" authorId="0" shapeId="0" xr:uid="{17BE59AF-FA15-498B-B9EA-135964EC1E24}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>DAÑO ACOPLE MANGUERA TERMOREGULADOR</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B18" authorId="0" shapeId="0" xr:uid="{7B260135-ACBC-49D8-8F8A-B4210B1BDA44}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Falta de dosis, revision carrusel de insercion</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C18" authorId="0" shapeId="0" xr:uid="{429362A1-CD6B-48B2-80DA-B2790AB57849}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revivion de carrusel de insercion alarma SQ18</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D18" authorId="0" shapeId="0" xr:uid="{7E188797-64DE-418F-96D2-F11206E705DC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>fuga de agua cavidad #16</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G18" authorId="0" shapeId="0" xr:uid="{9FDF6627-A5BB-41AC-90C6-0F6DB526E286}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>falla termoregulador temperatura alta</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C19" authorId="0" shapeId="0" xr:uid="{3BC30261-9595-4699-B7B6-324B85AA9A22}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revivion de carrusel de insercion alarma SQ18</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G19" authorId="0" shapeId="0" xr:uid="{66913330-8953-4480-A5D1-A0A3F8EA135E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>falla termoregulador temperatura alta</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B20" authorId="0" shapeId="0" xr:uid="{84AE15EC-3C6D-4562-8474-BF508912A9E7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revision motor centralita.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I20" authorId="0" shapeId="0" xr:uid="{A69585A2-B589-458C-98AE-1508D06C46D7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>1. punzon # 30 y 31 con humedad
+2. Humedad en punzones 30 y 31</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{74979DE9-95CB-4ECC-A616-F865906714EC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revision y cambio punzones posicion # 12 y # 16 presenta rechupe</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E22" authorId="0" shapeId="0" xr:uid="{3C01FAFE-D463-48A8-9E15-8852B56510FA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revision Cavidad y Punzon No 60 Por Golpe</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E23" authorId="0" shapeId="0" xr:uid="{1A258370-F031-4F8E-91A3-A23260D702C2}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revision Cavidad y Punzon No 60 Por Golpe</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F25" authorId="0" shapeId="0" xr:uid="{E6257C99-4332-4067-AF91-4A3B8DCEF294}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>1. revision punzon # 15 y 48 por golpe
+2. punzones golpeados</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I25" authorId="0" shapeId="0" xr:uid="{DFDD64E5-9F35-4DF7-88D3-0BE9DE17016E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alarma BQ8 en FSM y fallaBY-PASS</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B27" authorId="0" shapeId="0" xr:uid="{F4F98F93-3EA2-4731-BD35-E2F7ED87E3A4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Falla FSM de Sincronismo</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E29" authorId="0" shapeId="0" xr:uid="{48B614A7-0337-4487-B1E6-49565D514377}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>falla por alarma 3024 controla sp5v</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C30" authorId="0" shapeId="0" xr:uid="{888D479C-5EF7-4DA4-9856-136C0A3E0BDD}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>1. revision cavida 15 por fuga aceite, revision carrusel de insercion |por tapa doblada
+2. tapa golpeada, error sincronizacion
+3. Revisicion cavidad #15 por falla en la inspeccion del palley</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C31" authorId="0" shapeId="0" xr:uid="{C1F53E51-C14F-4A81-A047-EEA6EEE04AEC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Falla por sincronizacion en la fsm</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B32" authorId="0" shapeId="0" xr:uid="{0675B41E-0B35-45DC-A9F7-BE337743085B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revision fuga material tornillo estrusor</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D32" authorId="0" shapeId="0" xr:uid="{72D022AA-F049-4278-9A4A-866A56C0EEAE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Falta de grasa en la  FSM</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C33" authorId="0" shapeId="0" xr:uid="{144E8A99-C264-41F0-8B22-24F4094A318B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Parada por alarma BQ8 en la FSM</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F33" authorId="0" shapeId="0" xr:uid="{264489BA-3040-438F-B756-44A94576E6F8}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revision punzon y cavidad # 2 por golpe</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C34" authorId="0" shapeId="0" xr:uid="{750E5284-922C-48B0-BEAD-237E8A22A31F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Parada por alarma BQ8 en la FSM</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E36" authorId="0" shapeId="0" xr:uid="{1A273CBC-9CEA-45BF-936E-074DA1FAB9AE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Parada Por Leve Golpe Punzon No 5</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B37" authorId="0" shapeId="0" xr:uid="{24C55F1F-4FD1-4CA2-81C4-74B0201565AD}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revisar alarma SP19</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E37" authorId="0" shapeId="0" xr:uid="{810D403A-8D5D-4E27-B165-74D87C38B2D6}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>1. Punzon 46 posicion 5 concavidad alta.
+2. Revisionpunzon # 46 posicion # 5 por concavidad alta</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E38" authorId="0" shapeId="0" xr:uid="{16E8E5AA-4AFA-4406-A8EF-D6A397B9B3B6}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Revision punzones #43 - #41 por rebaba posicion #5 - #41</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C39" authorId="0" shapeId="0" xr:uid="{72718C13-8005-4CA3-8F24-F647B0763506}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>punzon # 4 por concavidad fuera de norma</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Diego</author>
+  </authors>
+  <commentList>
+    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{542D4147-110A-4D61-BB00-DAA3129C3B19}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mantenimiento preventivo trimestral</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B16" authorId="0" shapeId="0" xr:uid="{E947CA84-B256-416F-8061-DC99A096D0A1}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mantenimiento preventivo quincenal</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D17" authorId="0" shapeId="0" xr:uid="{DCDB2268-9595-48D8-860E-861D056CBE5D}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mantenimiento preventivo mensual</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G18" authorId="0" shapeId="0" xr:uid="{A4B41BC6-33BC-4721-A31A-E8D66DC84B02}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mantenimiento preventivo quincenal</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I24" authorId="0" shapeId="0" xr:uid="{A73ABBED-05AF-4A19-A1AC-1E6E3031B393}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mantenimiento preventivo mensual</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H25" authorId="0" shapeId="0" xr:uid="{98988BDF-DE47-4390-B498-F3DB94B00F47}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mantenimiento preventivo mensual</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F26" authorId="0" shapeId="0" xr:uid="{573E425F-F67C-42DA-A3D0-89DC4B0D4B57}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mantenimiento preventivo quincenal</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F37" authorId="0" shapeId="0" xr:uid="{5C35FE65-46B3-430B-8A9F-65D0B2A1769E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mantenimiento preventivo trimestral</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F38" authorId="0" shapeId="0" xr:uid="{E348B4EE-8156-4D65-BAAD-14826D8D6A73}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mantenimiento preventivo trimestral</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F39" authorId="0" shapeId="0" xr:uid="{87AC814A-B43C-42FB-ABB0-B5B6EA6D6AC7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mantenimiento preventivo trimestral</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F40" authorId="0" shapeId="0" xr:uid="{C05598B7-6D11-4647-99B3-0B30879C744D}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mantenimiento preventivo trimestral</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Diego</author>
+  </authors>
+  <commentList>
+    <comment ref="C19" authorId="0" shapeId="0" xr:uid="{135935B5-57E5-4519-A73D-0173AFB625D9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Cambio de referencia</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C20" authorId="0" shapeId="0" xr:uid="{2382DB2A-F918-499C-A6E6-4085F9394E8A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Cambio a tapa VIDRIO MCA</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{DCC5D6DC-1B5F-472C-8135-CCDE11E157F7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Cambio a tapa VIDRIO MCA</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C28" authorId="0" shapeId="0" xr:uid="{AA97CF00-B4F1-430B-A6DC-AAA8B0D2A966}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Cambio de referencia vidrio a PRB</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C35" authorId="0" shapeId="0" xr:uid="{D2B65331-321B-43E6-9095-D1B721D4AA53}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>1. Cambio de referencia de PET PRB a MCA vidrio
+2. cambio de referencia de PRB a VIDRIO</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="119">
   <si>
     <t xml:space="preserve">DÍA / planta </t>
   </si>
@@ -189,6 +1043,268 @@
   <si>
     <t>c</t>
   </si>
+  <si>
+    <t>Falla FSM de Sincronismo</t>
+  </si>
+  <si>
+    <t>Se Desmonta Encoder Carrussel de Corte, Se realiza Mantenimiento, Se Instala y se Sincroniza OK.</t>
+  </si>
+  <si>
+    <t>Falta de dosis, revision carrusel de insercion</t>
+  </si>
+  <si>
+    <t>Revision precarga de carrusel de insercion, ajuste y calibracion de cuchillas. Cambio esparrago de termoregulador de la puerta lado operador</t>
+  </si>
+  <si>
+    <t>Revision fuga material tornillo estrusor</t>
+  </si>
+  <si>
+    <t>Se realiza separacion de cañon con bridas de la bomba de la estrusora, posteriormente se realiza limpieza de material plastico que fugó, se cambia una terminal de bronce porque estaba dañada, se ensambla todo y se realiza seguimiento, no presenta mas fuga</t>
+  </si>
+  <si>
+    <t>Revision motor centralita.</t>
+  </si>
+  <si>
+    <t>se realiza revision y se cambia filtro de aceite motor queda consumiento 4,5 amp ok</t>
+  </si>
+  <si>
+    <t>Revision pantalla CVS - No prende</t>
+  </si>
+  <si>
+    <t>Se instala monitor. Queda funcionando</t>
+  </si>
+  <si>
+    <t>Revision calbibracion de cuchillas</t>
+  </si>
+  <si>
+    <t>Se recalibran las ocho cuchillas se cambia dos tornillos, se sugiere cambiar todos los tornillos para mejor ajuste a la cuchilla</t>
+  </si>
+  <si>
+    <t>Revisar alarma SP19</t>
+  </si>
+  <si>
+    <t>Se realiza desmontaje de filtro zona cavidades y se evidencia limpio, se ajusta flujometro</t>
+  </si>
+  <si>
+    <t>Parada por alarma BQ8 en la FSM</t>
+  </si>
+  <si>
+    <t>Se cambia acople araña del servomotor superior del carrusel de corte, se prueban encoder´s reparados y uno de ellos funciona y la maquina trabaja de 11 a 13:40 pero pierde el sincronismo y para volver a  arrancar la maquina toca sincronizar. al final se monta encoder nuevo que llego
+Se realiza sincronismo en FSM con la galgas y la maquina inicia ok</t>
+  </si>
+  <si>
+    <t>Falla por sincronizacion en la fsm</t>
+  </si>
+  <si>
+    <t>revision cavida 15 por fuga aceite, revision carrusel de insercion |por tapa doblada</t>
+  </si>
+  <si>
+    <t>Se realiza desmonte de cavidad y expulsor ademas se desmonta el punzon para realizar las respectivad calibraciones .Se sincoroniza la salida de la tapa de la termocompresora y la cfm con apoyo de Jhon Alexander Cacais</t>
+  </si>
+  <si>
+    <t>Revivion de carrusel de insercion alarma SQ18</t>
+  </si>
+  <si>
+    <t>Se realiza cambio de correas de transmision de carrusel de formado y carrusel de insercion</t>
+  </si>
+  <si>
+    <t>tapa golpeada, error sincronizacion</t>
+  </si>
+  <si>
+    <t>Entortamiento carrusel de insercion.</t>
+  </si>
+  <si>
+    <t>Se saca carrusel de insercion, algunas guardas y soportes pára poder cortar y sacar la torta</t>
+  </si>
+  <si>
+    <t>Revisicion cavidad #15 por falla en la inspeccion del palley</t>
+  </si>
+  <si>
+    <t>Se baja actuador #15, se encuentra buje bronce suelto, se aplica pegante roscas y se aprieta buje, se centra cavidad. Apoyo supervisor de produccion</t>
+  </si>
+  <si>
+    <t>Revision zonas boquilla y cuerpo casquilo se suben de temperatura por encima del set poin.</t>
+  </si>
+  <si>
+    <t>se realiza ajuste de conexiones del cableado de las termocuplas de esas zonas y se verifica que no este directo ningun SSR.</t>
+  </si>
+  <si>
+    <t>punzon # 4 por concavidad fuera de norma</t>
+  </si>
+  <si>
+    <t>se cambia regulador de aire punzon</t>
+  </si>
+  <si>
+    <t>Revision y cambio punzones posicion # 12 y # 16 presenta rechupe</t>
+  </si>
+  <si>
+    <t>Se realiza cambio de punzones de la posicion # 12  se deja elpunzon # 34 de respuesto y en la posicion # 16 se coloca el punzon de repuesto # 33.</t>
+  </si>
+  <si>
+    <t>alarma BQ8 encoder</t>
+  </si>
+  <si>
+    <t>Cambiar encoder carrusel en la FSM 3 Por que se paso para habilitar la FMS 5 CCM5</t>
+  </si>
+  <si>
+    <t>Se realiza limpieza interna de encoder se verican contactos internos del conector encoder se sincroniza y se habilita.</t>
+  </si>
+  <si>
+    <t>Bajar Encoder  Carrusel de Corte en la FSM 3</t>
+  </si>
+  <si>
+    <t>Temperatura alta en la zona de la bomba y fuga de agua cavidad 14.</t>
+  </si>
+  <si>
+    <t>Alarma SP20</t>
+  </si>
+  <si>
+    <t>Se desmonta filtro, se le realiza limpieza, se instala, se adiciona agua, queda ok.</t>
+  </si>
+  <si>
+    <t>BLOQUEO POR ALARMA CONTROLADOR SP20</t>
+  </si>
+  <si>
+    <t>se realiza mantenimiento al termoregulador, se verifican membranas, se limpian filtros. Queda ok se entrega a produccion.</t>
+  </si>
+  <si>
+    <t>Temperatura alta en la zona de la bomba y fuga de ahua cavidad 14.</t>
+  </si>
+  <si>
+    <t>se realiza desmonte de filtro de equipos auxiliares en termoreguador se limpia se  prueba ok</t>
+  </si>
+  <si>
+    <t>Falta de grasa en la  FSM</t>
+  </si>
+  <si>
+    <t>Se sube el nivel de la grasa en la FSM</t>
+  </si>
+  <si>
+    <t>fuga de agua cavidad #16</t>
+  </si>
+  <si>
+    <t>Se realiza cambio de mangueras de cavidad, se hace cebtrado de cavidad y montaje</t>
+  </si>
+  <si>
+    <t>Parada por alarma SP18</t>
+  </si>
+  <si>
+    <t>Se desmonta y se limpia filtro, despues se vuelte a montar</t>
+  </si>
+  <si>
+    <t>falla por alarma 3024 controla sp5v</t>
+  </si>
+  <si>
+    <t>se realiza cambio de bomba de vacio se instala la de la pmv 3 por autorizacion de edison solano se prueba ok</t>
+  </si>
+  <si>
+    <t>Revision Cavidad y Punzon No 60 Por Golpe</t>
+  </si>
+  <si>
+    <t>Se realiza cambio de punzon; el numero 60 se baja y se monta el 31, se cambia cavidad por una nueva</t>
+  </si>
+  <si>
+    <t>Revisionpunzon # 46 posicion # 5 por concavidad alta</t>
+  </si>
+  <si>
+    <t>Se cambia punzon por uno de repuesto</t>
+  </si>
+  <si>
+    <t>Parada Por Leve Golpe Punzon No 5</t>
+  </si>
+  <si>
+    <t>Se Reviza y se Cambia Punzon No 5 Posiscion No 5 Se Prueba OK.</t>
+  </si>
+  <si>
+    <t>Revision punzones #43 - #41 por rebaba posicion #5 - #41</t>
+  </si>
+  <si>
+    <t>Se realiza cambio de punzones #41 y #5</t>
+  </si>
+  <si>
+    <t>Punzon 46 posicion 5 concavidad alta.</t>
+  </si>
+  <si>
+    <t>FALLA SINCRONISMO CARRUSELES</t>
+  </si>
+  <si>
+    <t>Se Cambia Encoder, se Instala Encoder de la CCM 3 se Sincroniza Maquina, se Prueba OK.</t>
+  </si>
+  <si>
+    <t>punzones golpeados</t>
+  </si>
+  <si>
+    <t>revision punzon # 15 y 48 por golpe</t>
+  </si>
+  <si>
+    <t>se realiza cambio de punzon # 15 por desportillado y esjeco de cavidad golpeado, se realiza cambio de punzon # 48 por golpe se prueba ok</t>
+  </si>
+  <si>
+    <t>Revision punzon y cavidad # 2 por golpe</t>
+  </si>
+  <si>
+    <t>Se instala punzon IP 1415 y cabio de espejo posicion # 2.</t>
+  </si>
+  <si>
+    <t>PERDIDA DE SINCRONISMO FSM</t>
+  </si>
+  <si>
+    <t>ajuste de proceso, se baja la velocidad a la FSM a 800 tapas por minuto. Queda ok.</t>
+  </si>
+  <si>
+    <t>Sin descripción de parada</t>
+  </si>
+  <si>
+    <t>falla termoregulador temperatura alta</t>
+  </si>
+  <si>
+    <t>Se realiza cambio de manguera de entrada a termoregulador, se evidencia bobina suelta de la zona de punzones, se abren llaves de chiller arranca ok, se cambia UPS en FSM</t>
+  </si>
+  <si>
+    <t>tapa con anillo doblado recalentamiento en punzon</t>
+  </si>
+  <si>
+    <t>bloque de presion en tapa deformada refrigeracion en punzones defisiente</t>
+  </si>
+  <si>
+    <t>se realiza revision y se evidencia amarres en mangueras de recirculacion y se evidencia que de los punzones que montaron 1 tiene golpe se reakiza mtto de 1 punzon por parte de diego carvajas se monta se prueba ok</t>
+  </si>
+  <si>
+    <t>DAÑO ACOPLE MANGUERA TERMOREGULADOR</t>
+  </si>
+  <si>
+    <t>se desmosnta sistema de acople mangueras entrada agua chiller y se evidencia con fisura</t>
+  </si>
+  <si>
+    <t>Revision daño de racor punzon #39 (fuga de agua)</t>
+  </si>
+  <si>
+    <t>Se baja punzon y expulsor para limpieza de agua cambiar racor. Ensamblar pero continua el problema en cavidad 35 ala 41 se bajan punzones y expulsores, se realiza limpieza se monta, el problema continua. Se bajan nuevamente punzones del 35 al 40 se realiza mantenimiento cambio de empaques. montar nuevamente</t>
+  </si>
+  <si>
+    <t>fuga de agua</t>
+  </si>
+  <si>
+    <t>se corrige fuga</t>
+  </si>
+  <si>
+    <t>Alarma BQ8 en FSM y fallaBY-PASS</t>
+  </si>
+  <si>
+    <t>Se realiza inspeccion de funcionamiento de maquina, en modo manual despues de un tiempo pierde la lectura de encoder, se desmonta encoder y se hace el montaje de uno de pruebas pero no lo reconoce la maquina, se hace mntaje del ecoder desmontado, se hace ajuste de sincronismo arranca ok. Se requiere programar parada de maquina de 1 turno para mantenimiento de BY-.PASS</t>
+  </si>
+  <si>
+    <t>Humedad en punzones 30 y 31</t>
+  </si>
+  <si>
+    <t>Se realiza cambio de punzon #30 y 31</t>
+  </si>
+  <si>
+    <t>punzon # 30 y 31 con humedad</t>
+  </si>
+  <si>
+    <t>se realiza cambio de punzon 30 y 31 se pureba ok</t>
+  </si>
 </sst>
 </file>
 
@@ -199,7 +1315,7 @@
     <numFmt numFmtId="165" formatCode="h:mm:ss;@"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="36">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -412,6 +1528,13 @@
       <sz val="10"/>
       <color indexed="8"/>
       <name val="Arial monospaced for SAP"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1130,16 +2253,16 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -5017,19 +6140,19 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>120</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>300</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>225</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -5050,7 +6173,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0</c:v>
+                  <c:v>310</c:v>
                 </c:pt>
                 <c:pt idx="17">
                   <c:v>0</c:v>
@@ -5065,7 +6188,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0</c:v>
+                  <c:v>240</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>0</c:v>
@@ -5080,7 +6203,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="27">
                   <c:v>0</c:v>
@@ -5230,13 +6353,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>160</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>300</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -5245,16 +6368,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>265</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>70</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -5281,19 +6404,19 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0</c:v>
+                  <c:v>1105</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0</c:v>
+                  <c:v>645</c:v>
                 </c:pt>
                 <c:pt idx="21">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0</c:v>
+                  <c:v>757</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0</c:v>
+                  <c:v>350</c:v>
                 </c:pt>
                 <c:pt idx="24">
                   <c:v>0</c:v>
@@ -5308,7 +6431,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0</c:v>
+                  <c:v>70</c:v>
                 </c:pt>
                 <c:pt idx="29">
                   <c:v>0</c:v>
@@ -5452,22 +6575,22 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>740</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>670</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>380</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -5509,7 +6632,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0</c:v>
+                  <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>0</c:v>
@@ -5701,10 +6824,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0</c:v>
+                  <c:v>90</c:v>
                 </c:pt>
                 <c:pt idx="13">
                   <c:v>0</c:v>
@@ -5722,7 +6845,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="19">
                   <c:v>0</c:v>
@@ -5743,13 +6866,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0</c:v>
+                  <c:v>50</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0</c:v>
+                  <c:v>80</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0</c:v>
+                  <c:v>30</c:v>
                 </c:pt>
                 <c:pt idx="28">
                   <c:v>0</c:v>
@@ -5896,10 +7019,10 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>120</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>780</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -5932,7 +7055,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>495</c:v>
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>0</c:v>
@@ -5956,7 +7079,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0</c:v>
+                  <c:v>170</c:v>
                 </c:pt>
                 <c:pt idx="23">
                   <c:v>0</c:v>
@@ -6442,19 +7565,19 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>680</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>180</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>360</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>180</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -6548,7 +7671,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -6686,7 +7809,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>150</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -6701,7 +7824,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>200</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -7389,28 +8512,28 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1240</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>3902</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>2110</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>1565</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>1400</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>600</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>350</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -7738,7 +8861,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>220</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>0</c:v>
@@ -8185,7 +9308,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>360</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -8656,7 +9779,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>420</c:v>
                 </c:pt>
                 <c:pt idx="16">
                   <c:v>0</c:v>
@@ -8689,16 +9812,16 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0</c:v>
+                  <c:v>1320</c:v>
                 </c:pt>
                 <c:pt idx="27">
-                  <c:v>0</c:v>
+                  <c:v>1440</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>0</c:v>
+                  <c:v>1560</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>0</c:v>
+                  <c:v>1440</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9172,7 +10295,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -9305,7 +10428,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>410</c:v>
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>0</c:v>
@@ -9422,7 +10545,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>430</c:v>
                 </c:pt>
                 <c:pt idx="15">
                   <c:v>0</c:v>
@@ -10634,28 +11757,28 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>220</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>360</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>6960</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>480</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>410</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>430</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -11232,13 +12355,13 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>240</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>1440</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>225</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -11259,7 +12382,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0</c:v>
+                  <c:v>960</c:v>
                 </c:pt>
                 <c:pt idx="18">
                   <c:v>0</c:v>
@@ -11280,7 +12403,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0</c:v>
+                  <c:v>450</c:v>
                 </c:pt>
                 <c:pt idx="25">
                   <c:v>0</c:v>
@@ -13460,7 +14583,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>3315</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -33757,44 +34880,44 @@
       <c r="I147" s="17"/>
     </row>
     <row r="148" spans="1:9" ht="15.75" thickTop="1">
-      <c r="A148" s="129" t="s">
-        <v>0</v>
-      </c>
-      <c r="B148" s="129" t="s">
+      <c r="A148" s="131" t="s">
+        <v>0</v>
+      </c>
+      <c r="B148" s="131" t="s">
         <v>1</v>
       </c>
-      <c r="C148" s="129" t="s">
+      <c r="C148" s="131" t="s">
         <v>2</v>
       </c>
-      <c r="D148" s="129" t="s">
+      <c r="D148" s="131" t="s">
         <v>10</v>
       </c>
-      <c r="E148" s="129" t="s">
+      <c r="E148" s="131" t="s">
         <v>11</v>
       </c>
-      <c r="F148" s="129" t="s">
+      <c r="F148" s="131" t="s">
         <v>12</v>
       </c>
-      <c r="G148" s="129" t="s">
+      <c r="G148" s="131" t="s">
         <v>13</v>
       </c>
-      <c r="H148" s="129" t="s">
+      <c r="H148" s="131" t="s">
         <v>14</v>
       </c>
-      <c r="I148" s="129" t="s">
+      <c r="I148" s="131" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="149" spans="1:9" ht="15.75" thickBot="1">
-      <c r="A149" s="130"/>
-      <c r="B149" s="130"/>
-      <c r="C149" s="130"/>
-      <c r="D149" s="130"/>
-      <c r="E149" s="130"/>
-      <c r="F149" s="130"/>
-      <c r="G149" s="130"/>
-      <c r="H149" s="130"/>
-      <c r="I149" s="130"/>
+      <c r="A149" s="132"/>
+      <c r="B149" s="132"/>
+      <c r="C149" s="132"/>
+      <c r="D149" s="132"/>
+      <c r="E149" s="132"/>
+      <c r="F149" s="132"/>
+      <c r="G149" s="132"/>
+      <c r="H149" s="132"/>
+      <c r="I149" s="132"/>
     </row>
     <row r="150" spans="1:9" ht="21.75" thickTop="1">
       <c r="A150" s="18">
@@ -34736,44 +35859,44 @@
       <c r="I182" s="17"/>
     </row>
     <row r="183" spans="1:9" ht="15.75" thickTop="1">
-      <c r="A183" s="131" t="s">
-        <v>0</v>
-      </c>
-      <c r="B183" s="131" t="s">
+      <c r="A183" s="129" t="s">
+        <v>0</v>
+      </c>
+      <c r="B183" s="129" t="s">
         <v>1</v>
       </c>
-      <c r="C183" s="131" t="s">
+      <c r="C183" s="129" t="s">
         <v>2</v>
       </c>
-      <c r="D183" s="131" t="s">
+      <c r="D183" s="129" t="s">
         <v>10</v>
       </c>
-      <c r="E183" s="131" t="s">
+      <c r="E183" s="129" t="s">
         <v>11</v>
       </c>
-      <c r="F183" s="131" t="s">
+      <c r="F183" s="129" t="s">
         <v>12</v>
       </c>
-      <c r="G183" s="131" t="s">
+      <c r="G183" s="129" t="s">
         <v>13</v>
       </c>
-      <c r="H183" s="131" t="s">
+      <c r="H183" s="129" t="s">
         <v>14</v>
       </c>
-      <c r="I183" s="131" t="s">
+      <c r="I183" s="129" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="184" spans="1:9" ht="15.75" thickBot="1">
-      <c r="A184" s="132"/>
-      <c r="B184" s="132"/>
-      <c r="C184" s="132"/>
-      <c r="D184" s="132"/>
-      <c r="E184" s="132"/>
-      <c r="F184" s="132"/>
-      <c r="G184" s="132"/>
-      <c r="H184" s="132"/>
-      <c r="I184" s="132"/>
+      <c r="A184" s="130"/>
+      <c r="B184" s="130"/>
+      <c r="C184" s="130"/>
+      <c r="D184" s="130"/>
+      <c r="E184" s="130"/>
+      <c r="F184" s="130"/>
+      <c r="G184" s="130"/>
+      <c r="H184" s="130"/>
+      <c r="I184" s="130"/>
     </row>
     <row r="185" spans="1:9" ht="21.75" thickTop="1">
       <c r="A185" s="8">
@@ -37665,60 +38788,6 @@
     <row r="289" ht="15.75" thickTop="1"/>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G41:G42"/>
-    <mergeCell ref="H41:H42"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="B41:B42"/>
-    <mergeCell ref="C41:C42"/>
-    <mergeCell ref="D41:D42"/>
-    <mergeCell ref="E41:E42"/>
-    <mergeCell ref="F41:F42"/>
-    <mergeCell ref="F255:F256"/>
-    <mergeCell ref="G255:G256"/>
-    <mergeCell ref="H255:H256"/>
-    <mergeCell ref="A219:A220"/>
-    <mergeCell ref="B219:B220"/>
-    <mergeCell ref="C219:C220"/>
-    <mergeCell ref="D219:D220"/>
-    <mergeCell ref="E219:E220"/>
-    <mergeCell ref="F219:F220"/>
-    <mergeCell ref="A255:A256"/>
-    <mergeCell ref="B255:B256"/>
-    <mergeCell ref="C255:C256"/>
-    <mergeCell ref="D255:D256"/>
-    <mergeCell ref="E255:E256"/>
-    <mergeCell ref="F183:F184"/>
-    <mergeCell ref="G183:G184"/>
-    <mergeCell ref="H183:H184"/>
-    <mergeCell ref="I183:I184"/>
-    <mergeCell ref="G219:G220"/>
-    <mergeCell ref="H219:H220"/>
-    <mergeCell ref="A183:A184"/>
-    <mergeCell ref="B183:B184"/>
-    <mergeCell ref="C183:C184"/>
-    <mergeCell ref="D183:D184"/>
-    <mergeCell ref="E183:E184"/>
-    <mergeCell ref="H112:H113"/>
-    <mergeCell ref="I112:I113"/>
-    <mergeCell ref="A148:A149"/>
-    <mergeCell ref="B148:B149"/>
-    <mergeCell ref="C148:C149"/>
-    <mergeCell ref="D148:D149"/>
-    <mergeCell ref="E148:E149"/>
-    <mergeCell ref="F148:F149"/>
-    <mergeCell ref="G148:G149"/>
-    <mergeCell ref="H148:H149"/>
-    <mergeCell ref="I148:I149"/>
     <mergeCell ref="G76:G77"/>
     <mergeCell ref="H76:H77"/>
     <mergeCell ref="I76:I77"/>
@@ -37735,6 +38804,60 @@
     <mergeCell ref="D76:D77"/>
     <mergeCell ref="E76:E77"/>
     <mergeCell ref="F76:F77"/>
+    <mergeCell ref="H112:H113"/>
+    <mergeCell ref="I112:I113"/>
+    <mergeCell ref="A148:A149"/>
+    <mergeCell ref="B148:B149"/>
+    <mergeCell ref="C148:C149"/>
+    <mergeCell ref="D148:D149"/>
+    <mergeCell ref="E148:E149"/>
+    <mergeCell ref="F148:F149"/>
+    <mergeCell ref="G148:G149"/>
+    <mergeCell ref="H148:H149"/>
+    <mergeCell ref="I148:I149"/>
+    <mergeCell ref="A183:A184"/>
+    <mergeCell ref="B183:B184"/>
+    <mergeCell ref="C183:C184"/>
+    <mergeCell ref="D183:D184"/>
+    <mergeCell ref="E183:E184"/>
+    <mergeCell ref="F183:F184"/>
+    <mergeCell ref="G183:G184"/>
+    <mergeCell ref="H183:H184"/>
+    <mergeCell ref="I183:I184"/>
+    <mergeCell ref="G219:G220"/>
+    <mergeCell ref="H219:H220"/>
+    <mergeCell ref="F255:F256"/>
+    <mergeCell ref="G255:G256"/>
+    <mergeCell ref="H255:H256"/>
+    <mergeCell ref="A219:A220"/>
+    <mergeCell ref="B219:B220"/>
+    <mergeCell ref="C219:C220"/>
+    <mergeCell ref="D219:D220"/>
+    <mergeCell ref="E219:E220"/>
+    <mergeCell ref="F219:F220"/>
+    <mergeCell ref="A255:A256"/>
+    <mergeCell ref="B255:B256"/>
+    <mergeCell ref="C255:C256"/>
+    <mergeCell ref="D255:D256"/>
+    <mergeCell ref="E255:E256"/>
+    <mergeCell ref="G41:G42"/>
+    <mergeCell ref="H41:H42"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="A41:A42"/>
+    <mergeCell ref="B41:B42"/>
+    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="D41:D42"/>
+    <mergeCell ref="E41:E42"/>
+    <mergeCell ref="F41:F42"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:F6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -37810,38 +38933,68 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" thickTop="1">
-      <c r="A8" s="61"/>
-      <c r="B8" s="61"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="112"/>
+    <row r="8" spans="1:5" ht="41.25" thickTop="1">
+      <c r="A8" s="61">
+        <v>1</v>
+      </c>
+      <c r="B8" s="61" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" s="61" t="s">
+        <v>103</v>
+      </c>
+      <c r="D8" s="112">
+        <v>540</v>
+      </c>
       <c r="E8" s="122">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="61"/>
-      <c r="B9" s="71"/>
+      <c r="A9" s="61">
+        <v>2</v>
+      </c>
+      <c r="B9" s="71" t="s">
+        <v>104</v>
+      </c>
       <c r="C9" s="102"/>
-      <c r="D9" s="109"/>
+      <c r="D9" s="109">
+        <v>480</v>
+      </c>
       <c r="E9" s="123">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="61"/>
-      <c r="B10" s="71"/>
-      <c r="C10" s="79"/>
-      <c r="D10" s="109"/>
+    <row r="10" spans="1:5" ht="54">
+      <c r="A10" s="61">
+        <v>3</v>
+      </c>
+      <c r="B10" s="71" t="s">
+        <v>105</v>
+      </c>
+      <c r="C10" s="79" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" s="109">
+        <v>200</v>
+      </c>
       <c r="E10" s="124">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="61"/>
-      <c r="B11" s="71"/>
-      <c r="C11" s="102"/>
-      <c r="D11" s="109"/>
+    <row r="11" spans="1:5" ht="27">
+      <c r="A11" s="61">
+        <v>4</v>
+      </c>
+      <c r="B11" s="71" t="s">
+        <v>107</v>
+      </c>
+      <c r="C11" s="102" t="s">
+        <v>108</v>
+      </c>
+      <c r="D11" s="109">
+        <v>180</v>
+      </c>
       <c r="E11" s="125">
         <v>1</v>
       </c>
@@ -37851,18 +39004,14 @@
       <c r="B12" s="71"/>
       <c r="C12" s="71"/>
       <c r="D12" s="109"/>
-      <c r="E12" s="126">
-        <v>1</v>
-      </c>
+      <c r="E12" s="126"/>
     </row>
     <row r="13" spans="1:5" ht="17.25" customHeight="1">
       <c r="A13" s="61"/>
       <c r="B13" s="79"/>
       <c r="C13" s="104"/>
       <c r="D13" s="113"/>
-      <c r="E13" s="124">
-        <v>1</v>
-      </c>
+      <c r="E13" s="124"/>
     </row>
     <row r="14" spans="1:5" ht="17.25" customHeight="1">
       <c r="A14" s="61"/>
@@ -37897,8 +39046,8 @@
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
       <c r="D18" s="7">
-        <f>SUM(D8:D17)</f>
-        <v>0</v>
+        <f>SUM(D8:D11)</f>
+        <v>1400</v>
       </c>
       <c r="E18" s="4"/>
     </row>
@@ -38034,20 +39183,36 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" thickTop="1">
-      <c r="A8" s="61"/>
-      <c r="B8" s="61"/>
-      <c r="C8" s="103"/>
-      <c r="D8" s="117"/>
+    <row r="8" spans="1:5" ht="54.75" thickTop="1">
+      <c r="A8" s="61">
+        <v>1</v>
+      </c>
+      <c r="B8" s="61" t="s">
+        <v>109</v>
+      </c>
+      <c r="C8" s="103" t="s">
+        <v>110</v>
+      </c>
+      <c r="D8" s="117">
+        <v>480</v>
+      </c>
       <c r="E8" s="116">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="83">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="83"/>
-      <c r="B9" s="65"/>
-      <c r="C9" s="65"/>
-      <c r="D9" s="118"/>
+      <c r="B9" s="65" t="s">
+        <v>111</v>
+      </c>
+      <c r="C9" s="65" t="s">
+        <v>112</v>
+      </c>
+      <c r="D9" s="118">
+        <v>120</v>
+      </c>
       <c r="E9" s="116">
         <v>1</v>
       </c>
@@ -38113,8 +39278,8 @@
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
       <c r="D18" s="7">
-        <f>SUM(D8:D16)</f>
-        <v>0</v>
+        <f>SUM(D8:D9)</f>
+        <v>600</v>
       </c>
       <c r="E18" s="4"/>
     </row>
@@ -38253,28 +39418,56 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" thickTop="1">
-      <c r="A8" s="62"/>
-      <c r="B8" s="71"/>
-      <c r="C8" s="71"/>
-      <c r="D8" s="109"/>
+    <row r="8" spans="1:5" ht="68.25" thickTop="1">
+      <c r="A8" s="62">
+        <v>1</v>
+      </c>
+      <c r="B8" s="71" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" s="71" t="s">
+        <v>114</v>
+      </c>
+      <c r="D8" s="109">
+        <v>200</v>
+      </c>
       <c r="E8" s="116">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="62"/>
-      <c r="B9" s="71"/>
-      <c r="C9" s="71"/>
-      <c r="D9" s="71"/>
-      <c r="E9" s="83"/>
+      <c r="A9" s="62">
+        <v>2</v>
+      </c>
+      <c r="B9" s="71" t="s">
+        <v>115</v>
+      </c>
+      <c r="C9" s="71" t="s">
+        <v>116</v>
+      </c>
+      <c r="D9" s="71">
+        <v>75</v>
+      </c>
+      <c r="E9" s="83">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="62"/>
-      <c r="B10" s="71"/>
-      <c r="C10" s="71"/>
-      <c r="D10" s="71"/>
-      <c r="E10" s="83"/>
+      <c r="A10" s="62">
+        <v>3</v>
+      </c>
+      <c r="B10" s="71" t="s">
+        <v>117</v>
+      </c>
+      <c r="C10" s="71" t="s">
+        <v>118</v>
+      </c>
+      <c r="D10" s="71">
+        <v>75</v>
+      </c>
+      <c r="E10" s="83">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="62"/>
@@ -38323,8 +39516,8 @@
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
       <c r="D17" s="7">
-        <f>SUM(D8:D15)</f>
-        <v>0</v>
+        <f>SUM(D8:D10)</f>
+        <v>350</v>
       </c>
       <c r="E17" s="4"/>
     </row>
@@ -38471,7 +39664,7 @@
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="7">
-        <f>SUM(D8:D13)</f>
+        <f>SUM(D8:D8)</f>
         <v>0</v>
       </c>
     </row>
@@ -38580,7 +39773,7 @@
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
       <c r="D16" s="7">
-        <f>SUM(D8:D15)</f>
+        <f>SUM(D8:D8)</f>
         <v>0</v>
       </c>
     </row>
@@ -38609,7 +39802,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Hoja3"/>
   <dimension ref="A1:Q49"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
@@ -38634,7 +39827,7 @@
       <c r="G7" s="25"/>
     </row>
     <row r="8" spans="1:17" ht="19.5" customHeight="1" thickTop="1">
-      <c r="A8" s="131" t="s">
+      <c r="A8" s="129" t="s">
         <v>0</v>
       </c>
       <c r="B8" s="133" t="s">
@@ -38669,7 +39862,7 @@
       </c>
     </row>
     <row r="9" spans="1:17" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A9" s="132"/>
+      <c r="A9" s="130"/>
       <c r="B9" s="134"/>
       <c r="C9" s="134"/>
       <c r="D9" s="134"/>
@@ -38707,7 +39900,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="50">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="I10" s="50">
         <v>0</v>
@@ -38800,22 +39993,22 @@
         <v>0</v>
       </c>
       <c r="C13" s="50">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="D13" s="50">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="E13" s="50">
         <v>0</v>
       </c>
       <c r="F13" s="50">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="G13" s="50">
         <v>0</v>
       </c>
       <c r="H13" s="50">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="I13" s="50">
         <v>0</v>
@@ -38836,16 +40029,16 @@
         <v>0</v>
       </c>
       <c r="C14" s="50">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="D14" s="50">
-        <v>0</v>
+        <v>740</v>
       </c>
       <c r="E14" s="50">
         <v>0</v>
       </c>
       <c r="F14" s="50">
-        <v>0</v>
+        <v>780</v>
       </c>
       <c r="G14" s="50">
         <v>0</v>
@@ -38872,10 +40065,10 @@
         <v>0</v>
       </c>
       <c r="C15" s="50">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="D15" s="50">
-        <v>0</v>
+        <v>670</v>
       </c>
       <c r="E15" s="50">
         <v>0</v>
@@ -38884,7 +40077,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="50">
-        <v>0</v>
+        <v>680</v>
       </c>
       <c r="H15" s="50">
         <v>0</v>
@@ -38905,13 +40098,13 @@
         <v>46177</v>
       </c>
       <c r="B16" s="50">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="C16" s="50">
         <v>0</v>
       </c>
       <c r="D16" s="50">
-        <v>0</v>
+        <v>380</v>
       </c>
       <c r="E16" s="50">
         <v>0</v>
@@ -38941,7 +40134,7 @@
         <v>46178</v>
       </c>
       <c r="B17" s="50">
-        <v>0</v>
+        <v>120</v>
       </c>
       <c r="C17" s="50">
         <v>0</v>
@@ -38956,7 +40149,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="50">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="H17" s="50">
         <v>0</v>
@@ -38977,13 +40170,13 @@
         <v>46179</v>
       </c>
       <c r="B18" s="50">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="C18" s="50">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="D18" s="50">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E18" s="50">
         <v>0</v>
@@ -38992,7 +40185,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="50">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="H18" s="50">
         <v>0</v>
@@ -39016,7 +40209,7 @@
         <v>0</v>
       </c>
       <c r="C19" s="50">
-        <v>0</v>
+        <v>265</v>
       </c>
       <c r="D19" s="50">
         <v>0</v>
@@ -39028,7 +40221,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="50">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="H19" s="50">
         <v>0</v>
@@ -39049,7 +40242,7 @@
         <v>46181</v>
       </c>
       <c r="B20" s="50">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="C20" s="50">
         <v>0</v>
@@ -39070,7 +40263,7 @@
         <v>0</v>
       </c>
       <c r="I20" s="50">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="J20" s="50">
         <v>0</v>
@@ -39088,7 +40281,7 @@
         <v>0</v>
       </c>
       <c r="C21" s="50">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="D21" s="50">
         <v>0</v>
@@ -39130,7 +40323,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="50">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F22" s="50">
         <v>0</v>
@@ -39166,7 +40359,7 @@
         <v>0</v>
       </c>
       <c r="E23" s="50">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F23" s="50">
         <v>0</v>
@@ -39241,7 +40434,7 @@
         <v>0</v>
       </c>
       <c r="F25" s="50">
-        <v>0</v>
+        <v>495</v>
       </c>
       <c r="G25" s="50">
         <v>0</v>
@@ -39250,7 +40443,7 @@
         <v>0</v>
       </c>
       <c r="I25" s="50">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="J25" s="50">
         <v>0</v>
@@ -39301,7 +40494,7 @@
         <v>46188</v>
       </c>
       <c r="B27" s="50">
-        <v>0</v>
+        <v>310</v>
       </c>
       <c r="C27" s="50">
         <v>0</v>
@@ -39382,7 +40575,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="50">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F29" s="50">
         <v>0</v>
@@ -39412,7 +40605,7 @@
         <v>0</v>
       </c>
       <c r="C30" s="50">
-        <v>0</v>
+        <v>1105</v>
       </c>
       <c r="D30" s="50">
         <v>0</v>
@@ -39448,7 +40641,7 @@
         <v>0</v>
       </c>
       <c r="C31" s="50">
-        <v>0</v>
+        <v>645</v>
       </c>
       <c r="D31" s="50">
         <v>0</v>
@@ -39481,13 +40674,13 @@
         <v>46193</v>
       </c>
       <c r="B32" s="50">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="C32" s="50">
         <v>0</v>
       </c>
       <c r="D32" s="50">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E32" s="50">
         <v>0</v>
@@ -39520,7 +40713,7 @@
         <v>0</v>
       </c>
       <c r="C33" s="50">
-        <v>0</v>
+        <v>757</v>
       </c>
       <c r="D33" s="50">
         <v>0</v>
@@ -39529,7 +40722,7 @@
         <v>0</v>
       </c>
       <c r="F33" s="50">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="G33" s="50">
         <v>0</v>
@@ -39556,7 +40749,7 @@
         <v>0</v>
       </c>
       <c r="C34" s="50">
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="D34" s="50">
         <v>0</v>
@@ -39634,7 +40827,7 @@
         <v>0</v>
       </c>
       <c r="E36" s="50">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F36" s="50">
         <v>0</v>
@@ -39661,7 +40854,7 @@
         <v>46198</v>
       </c>
       <c r="B37" s="50">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C37" s="50">
         <v>0</v>
@@ -39670,7 +40863,7 @@
         <v>0</v>
       </c>
       <c r="E37" s="50">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F37" s="50">
         <v>0</v>
@@ -39706,7 +40899,7 @@
         <v>0</v>
       </c>
       <c r="E38" s="50">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F38" s="50">
         <v>0</v>
@@ -39736,7 +40929,7 @@
         <v>0</v>
       </c>
       <c r="C39" s="50">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="D39" s="50">
         <v>0</v>
@@ -39804,35 +40997,35 @@
       <c r="A41" s="13"/>
       <c r="B41" s="14">
         <f t="shared" ref="B41:K41" si="0">SUM(B10:B40)</f>
-        <v>0</v>
+        <v>1240</v>
       </c>
       <c r="C41" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3902</v>
       </c>
       <c r="D41" s="14">
         <f>SUM(D10:D40)</f>
-        <v>0</v>
+        <v>2110</v>
       </c>
       <c r="E41" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="F41" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1565</v>
       </c>
       <c r="G41" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="H41" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="I41" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="J41" s="14">
         <f t="shared" si="0"/>
@@ -39844,7 +41037,7 @@
       </c>
       <c r="L41" s="46">
         <f>SUM(B41:K41)</f>
-        <v>0</v>
+        <v>11647</v>
       </c>
     </row>
     <row r="42" spans="1:17" ht="19.5" thickTop="1">
@@ -39916,6 +41109,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="12">
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
     <mergeCell ref="F8:F9"/>
     <mergeCell ref="L9:N9"/>
     <mergeCell ref="J8:J9"/>
@@ -39923,11 +41121,6 @@
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="H8:H9"/>
     <mergeCell ref="I8:I9"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
@@ -39946,11 +41139,12 @@
   <pageSetup scale="80" orientation="landscape" verticalDpi="200" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:N52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
@@ -39976,52 +41170,52 @@
       <c r="G7" s="25"/>
     </row>
     <row r="8" spans="1:14" ht="19.5" customHeight="1" thickTop="1">
-      <c r="A8" s="131" t="s">
-        <v>0</v>
-      </c>
-      <c r="B8" s="131" t="s">
+      <c r="A8" s="129" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="129" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="131" t="s">
+      <c r="C8" s="129" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="131" t="s">
+      <c r="D8" s="129" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="131" t="s">
+      <c r="E8" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="131" t="s">
+      <c r="F8" s="129" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="131" t="s">
+      <c r="G8" s="129" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="131" t="s">
+      <c r="H8" s="129" t="s">
         <v>22</v>
       </c>
-      <c r="I8" s="131" t="s">
+      <c r="I8" s="129" t="s">
         <v>23</v>
       </c>
-      <c r="J8" s="131" t="s">
+      <c r="J8" s="129" t="s">
         <v>24</v>
       </c>
-      <c r="K8" s="131" t="s">
+      <c r="K8" s="129" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A9" s="132"/>
-      <c r="B9" s="132"/>
-      <c r="C9" s="132"/>
-      <c r="D9" s="132"/>
-      <c r="E9" s="132"/>
-      <c r="F9" s="132"/>
-      <c r="G9" s="132"/>
-      <c r="H9" s="132"/>
-      <c r="I9" s="132"/>
-      <c r="J9" s="132"/>
-      <c r="K9" s="132"/>
+      <c r="A9" s="130"/>
+      <c r="B9" s="130"/>
+      <c r="C9" s="130"/>
+      <c r="D9" s="130"/>
+      <c r="E9" s="130"/>
+      <c r="F9" s="130"/>
+      <c r="G9" s="130"/>
+      <c r="H9" s="130"/>
+      <c r="I9" s="130"/>
+      <c r="J9" s="130"/>
+      <c r="K9" s="130"/>
       <c r="L9" s="135"/>
       <c r="M9" s="135"/>
       <c r="N9" s="135"/>
@@ -40043,7 +41237,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="57">
-        <v>0</v>
+        <v>780</v>
       </c>
       <c r="G10" s="57">
         <v>0</v>
@@ -40241,7 +41435,7 @@
         <v>46177</v>
       </c>
       <c r="B16" s="57">
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="C16" s="57">
         <v>0</v>
@@ -40282,7 +41476,7 @@
         <v>0</v>
       </c>
       <c r="D17" s="57">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="E17" s="57">
         <v>0</v>
@@ -40326,7 +41520,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="57">
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="H18" s="57">
         <v>0</v>
@@ -40542,7 +41736,7 @@
         <v>0</v>
       </c>
       <c r="I24" s="57">
-        <v>0</v>
+        <v>430</v>
       </c>
       <c r="J24" s="57">
         <v>0</v>
@@ -40574,7 +41768,7 @@
         <v>0</v>
       </c>
       <c r="H25" s="57">
-        <v>0</v>
+        <v>410</v>
       </c>
       <c r="I25" s="57">
         <v>0</v>
@@ -40603,7 +41797,7 @@
         <v>0</v>
       </c>
       <c r="F26" s="57">
-        <v>0</v>
+        <v>420</v>
       </c>
       <c r="G26" s="57">
         <v>0</v>
@@ -40988,7 +42182,7 @@
         <v>0</v>
       </c>
       <c r="F37" s="57">
-        <v>0</v>
+        <v>1320</v>
       </c>
       <c r="G37" s="57">
         <v>0</v>
@@ -41023,7 +42217,7 @@
         <v>0</v>
       </c>
       <c r="F38" s="57">
-        <v>0</v>
+        <v>1440</v>
       </c>
       <c r="G38" s="57">
         <v>0</v>
@@ -41058,7 +42252,7 @@
         <v>0</v>
       </c>
       <c r="F39" s="57">
-        <v>0</v>
+        <v>1560</v>
       </c>
       <c r="G39" s="57">
         <v>0</v>
@@ -41093,7 +42287,7 @@
         <v>0</v>
       </c>
       <c r="F40" s="57">
-        <v>0</v>
+        <v>1440</v>
       </c>
       <c r="G40" s="57">
         <v>0</v>
@@ -41221,7 +42415,7 @@
       <c r="A44" s="13"/>
       <c r="B44" s="14">
         <f t="shared" ref="B44:K44" si="0">SUM(B10:B43)</f>
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="C44" s="14">
         <f t="shared" si="0"/>
@@ -41229,7 +42423,7 @@
       </c>
       <c r="D44" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="E44" s="14">
         <f t="shared" si="0"/>
@@ -41237,19 +42431,19 @@
       </c>
       <c r="F44" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>6960</v>
       </c>
       <c r="G44" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>480</v>
       </c>
       <c r="H44" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>410</v>
       </c>
       <c r="I44" s="14">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>430</v>
       </c>
       <c r="J44" s="14">
         <f t="shared" si="0"/>
@@ -41261,7 +42455,7 @@
       </c>
       <c r="L44" s="46">
         <f>SUM(B44:K44)</f>
-        <v>0</v>
+        <v>8860</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="32.25" customHeight="1" thickTop="1">
@@ -41333,6 +42527,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="12">
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
     <mergeCell ref="F8:F9"/>
     <mergeCell ref="L9:N9"/>
     <mergeCell ref="G8:G9"/>
@@ -41340,21 +42539,17 @@
     <mergeCell ref="J8:J9"/>
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="I8:I9"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup scale="80" orientation="landscape" verticalDpi="200" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
@@ -41378,52 +42573,52 @@
       <c r="G7" s="25"/>
     </row>
     <row r="8" spans="1:14" ht="19.5" customHeight="1" thickTop="1">
-      <c r="A8" s="131" t="s">
-        <v>0</v>
-      </c>
-      <c r="B8" s="131" t="s">
+      <c r="A8" s="129" t="s">
+        <v>0</v>
+      </c>
+      <c r="B8" s="129" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="131" t="s">
+      <c r="C8" s="129" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="131" t="s">
+      <c r="D8" s="129" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="131" t="s">
+      <c r="E8" s="129" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="131" t="s">
+      <c r="F8" s="129" t="s">
         <v>20</v>
       </c>
-      <c r="G8" s="131" t="s">
+      <c r="G8" s="129" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="131" t="s">
+      <c r="H8" s="129" t="s">
         <v>22</v>
       </c>
-      <c r="I8" s="131" t="s">
+      <c r="I8" s="129" t="s">
         <v>23</v>
       </c>
-      <c r="J8" s="131" t="s">
+      <c r="J8" s="129" t="s">
         <v>24</v>
       </c>
-      <c r="K8" s="131" t="s">
+      <c r="K8" s="129" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A9" s="132"/>
-      <c r="B9" s="132"/>
-      <c r="C9" s="132"/>
-      <c r="D9" s="132"/>
-      <c r="E9" s="132"/>
-      <c r="F9" s="132"/>
-      <c r="G9" s="132"/>
-      <c r="H9" s="132"/>
-      <c r="I9" s="132"/>
-      <c r="J9" s="132"/>
-      <c r="K9" s="132"/>
+      <c r="A9" s="130"/>
+      <c r="B9" s="130"/>
+      <c r="C9" s="130"/>
+      <c r="D9" s="130"/>
+      <c r="E9" s="130"/>
+      <c r="F9" s="130"/>
+      <c r="G9" s="130"/>
+      <c r="H9" s="130"/>
+      <c r="I9" s="130"/>
+      <c r="J9" s="130"/>
+      <c r="K9" s="130"/>
       <c r="L9" s="135"/>
       <c r="M9" s="135"/>
       <c r="N9" s="135"/>
@@ -41751,7 +42946,7 @@
         <v>0</v>
       </c>
       <c r="C19" s="57">
-        <v>0</v>
+        <v>240</v>
       </c>
       <c r="D19" s="57">
         <v>0</v>
@@ -41786,7 +42981,7 @@
         <v>0</v>
       </c>
       <c r="C20" s="57">
-        <v>0</v>
+        <v>1440</v>
       </c>
       <c r="D20" s="57">
         <v>0</v>
@@ -41821,7 +43016,7 @@
         <v>0</v>
       </c>
       <c r="C21" s="57">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="D21" s="57">
         <v>0</v>
@@ -42066,7 +43261,7 @@
         <v>0</v>
       </c>
       <c r="C28" s="57">
-        <v>0</v>
+        <v>960</v>
       </c>
       <c r="D28" s="57">
         <v>0</v>
@@ -42311,7 +43506,7 @@
         <v>0</v>
       </c>
       <c r="C35" s="57">
-        <v>0</v>
+        <v>450</v>
       </c>
       <c r="D35" s="57">
         <v>0</v>
@@ -42591,7 +43786,7 @@
       </c>
       <c r="C43" s="14">
         <f>SUM(C10:C42)</f>
-        <v>0</v>
+        <v>3315</v>
       </c>
       <c r="D43" s="14">
         <f t="shared" si="0"/>
@@ -42627,7 +43822,7 @@
       </c>
       <c r="L43" s="53">
         <f>SUM(B43:K43)</f>
-        <v>0</v>
+        <v>3315</v>
       </c>
     </row>
     <row r="44" spans="1:12" ht="19.5" thickTop="1">
@@ -42699,6 +43894,11 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="12">
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
     <mergeCell ref="F8:F9"/>
     <mergeCell ref="L9:N9"/>
     <mergeCell ref="G8:G9"/>
@@ -42706,16 +43906,12 @@
     <mergeCell ref="J8:J9"/>
     <mergeCell ref="K8:K9"/>
     <mergeCell ref="I8:I9"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup scale="80" orientation="landscape" verticalDpi="200" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -42753,54 +43949,124 @@
       </c>
       <c r="G7" s="32"/>
     </row>
-    <row r="8" spans="1:7" ht="15.75" thickTop="1">
-      <c r="A8" s="106"/>
-      <c r="B8" s="59"/>
-      <c r="C8" s="97"/>
-      <c r="D8" s="121"/>
-      <c r="E8" s="105"/>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="107"/>
-      <c r="B9" s="59"/>
-      <c r="C9" s="97"/>
-      <c r="D9" s="121"/>
-      <c r="E9" s="105"/>
+    <row r="8" spans="1:7" ht="27.75" thickTop="1">
+      <c r="A8" s="106">
+        <v>1</v>
+      </c>
+      <c r="B8" s="59" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="97" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="121">
+        <v>310</v>
+      </c>
+      <c r="E8" s="105">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="40.5">
+      <c r="A9" s="107">
+        <v>2</v>
+      </c>
+      <c r="B9" s="59" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="97" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="121">
+        <v>300</v>
+      </c>
+      <c r="E9" s="105">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:7" ht="22.5" customHeight="1">
-      <c r="A10" s="107"/>
-      <c r="B10" s="59"/>
-      <c r="C10" s="88"/>
-      <c r="D10" s="121"/>
-      <c r="E10" s="105"/>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="106"/>
-      <c r="B11" s="59"/>
-      <c r="C11" s="97"/>
-      <c r="D11" s="121"/>
-      <c r="E11" s="105"/>
+      <c r="A10" s="107">
+        <v>3</v>
+      </c>
+      <c r="B10" s="59" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="88" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="121">
+        <v>240</v>
+      </c>
+      <c r="E10" s="105">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="27">
+      <c r="A11" s="106">
+        <v>4</v>
+      </c>
+      <c r="B11" s="59" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="97" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="121">
+        <v>225</v>
+      </c>
+      <c r="E11" s="105">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="63"/>
-      <c r="B12" s="59"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="91"/>
-      <c r="E12" s="62"/>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="63"/>
-      <c r="B13" s="59"/>
-      <c r="C13" s="60"/>
-      <c r="D13" s="61"/>
-      <c r="E13" s="62"/>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="63"/>
-      <c r="B14" s="59"/>
-      <c r="C14" s="60"/>
-      <c r="D14" s="61"/>
-      <c r="E14" s="62"/>
+      <c r="A12" s="63">
+        <v>5</v>
+      </c>
+      <c r="B12" s="59" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="60" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="91">
+        <v>120</v>
+      </c>
+      <c r="E12" s="62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="40.5">
+      <c r="A13" s="63">
+        <v>6</v>
+      </c>
+      <c r="B13" s="59" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="60" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="61">
+        <v>25</v>
+      </c>
+      <c r="E13" s="62">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="27">
+      <c r="A14" s="63">
+        <v>7</v>
+      </c>
+      <c r="B14" s="59" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" s="60" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="61">
+        <v>20</v>
+      </c>
+      <c r="E14" s="62">
+        <v>1</v>
+      </c>
       <c r="F14"/>
       <c r="G14"/>
     </row>
@@ -42858,8 +44124,8 @@
       <c r="B22" s="40"/>
       <c r="C22" s="40"/>
       <c r="D22" s="41">
-        <f>SUM(D8:D20)</f>
-        <v>0</v>
+        <f>SUM(D8:D14)</f>
+        <v>1240</v>
       </c>
       <c r="E22" s="39"/>
     </row>
@@ -42941,79 +44207,173 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" thickTop="1">
-      <c r="A8" s="58"/>
-      <c r="B8" s="71"/>
-      <c r="C8" s="71"/>
-      <c r="D8" s="109"/>
+    <row r="8" spans="1:5" ht="95.25" thickTop="1">
+      <c r="A8" s="58">
+        <v>1</v>
+      </c>
+      <c r="B8" s="71" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="71" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="109">
+        <v>1107</v>
+      </c>
       <c r="E8" s="108">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="58"/>
-      <c r="B9" s="71"/>
+      <c r="A9" s="58">
+        <v>2</v>
+      </c>
+      <c r="B9" s="71" t="s">
+        <v>48</v>
+      </c>
       <c r="C9" s="71"/>
-      <c r="D9" s="109"/>
+      <c r="D9" s="109">
+        <v>645</v>
+      </c>
       <c r="E9" s="108">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="58"/>
-      <c r="B10" s="71"/>
-      <c r="C10" s="71"/>
-      <c r="D10" s="72"/>
-      <c r="E10" s="73"/>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="58"/>
-      <c r="B11" s="79"/>
-      <c r="C11" s="71"/>
-      <c r="D11" s="72"/>
-      <c r="E11" s="73"/>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="74"/>
-      <c r="B12" s="79"/>
-      <c r="C12" s="71"/>
-      <c r="D12" s="72"/>
-      <c r="E12" s="73"/>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" s="74"/>
-      <c r="B13" s="71"/>
-      <c r="C13" s="64"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="73"/>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" s="74"/>
-      <c r="B14" s="71"/>
-      <c r="C14" s="71"/>
-      <c r="D14" s="72"/>
-      <c r="E14" s="73"/>
-    </row>
-    <row r="15" spans="1:5">
-      <c r="A15" s="74"/>
-      <c r="B15" s="71"/>
-      <c r="C15" s="71"/>
-      <c r="D15" s="72"/>
-      <c r="E15" s="73"/>
+    <row r="10" spans="1:5" ht="54">
+      <c r="A10" s="58">
+        <v>3</v>
+      </c>
+      <c r="B10" s="71" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="71" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="72">
+        <v>470</v>
+      </c>
+      <c r="E10" s="73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="27">
+      <c r="A11" s="58">
+        <v>4</v>
+      </c>
+      <c r="B11" s="79" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="71" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="72">
+        <v>415</v>
+      </c>
+      <c r="E11" s="73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="27">
+      <c r="A12" s="74">
+        <v>5</v>
+      </c>
+      <c r="B12" s="79" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="71" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="72">
+        <v>395</v>
+      </c>
+      <c r="E12" s="73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="27">
+      <c r="A13" s="74">
+        <v>6</v>
+      </c>
+      <c r="B13" s="71" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="64" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="72">
+        <v>330</v>
+      </c>
+      <c r="E13" s="73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="40.5">
+      <c r="A14" s="74">
+        <v>7</v>
+      </c>
+      <c r="B14" s="71" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="71" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="72">
+        <v>240</v>
+      </c>
+      <c r="E14" s="73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="40.5">
+      <c r="A15" s="74">
+        <v>8</v>
+      </c>
+      <c r="B15" s="71" t="s">
+        <v>58</v>
+      </c>
+      <c r="C15" s="71" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="72">
+        <v>160</v>
+      </c>
+      <c r="E15" s="73">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="74"/>
-      <c r="B16" s="71"/>
-      <c r="C16" s="71"/>
-      <c r="D16" s="72"/>
-      <c r="E16" s="73"/>
-    </row>
-    <row r="17" spans="1:5">
-      <c r="A17" s="74"/>
-      <c r="B17" s="71"/>
-      <c r="C17" s="71"/>
-      <c r="D17" s="72"/>
-      <c r="E17" s="73"/>
+      <c r="A16" s="74">
+        <v>9</v>
+      </c>
+      <c r="B16" s="71" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="71" t="s">
+        <v>61</v>
+      </c>
+      <c r="D16" s="72">
+        <v>70</v>
+      </c>
+      <c r="E16" s="73">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="40.5">
+      <c r="A17" s="74">
+        <v>10</v>
+      </c>
+      <c r="B17" s="71" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="71" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" s="72">
+        <v>70</v>
+      </c>
+      <c r="E17" s="73">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="74"/>
@@ -43048,8 +44408,8 @@
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
       <c r="D23" s="7">
-        <f>SUM(D8:D22)</f>
-        <v>0</v>
+        <f>SUM(D8:D17)</f>
+        <v>3902</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="15.75" thickTop="1"/>
@@ -43107,83 +44467,169 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.75" thickTop="1">
-      <c r="A8" s="75"/>
-      <c r="B8" s="65"/>
+      <c r="A8" s="75">
+        <v>1</v>
+      </c>
+      <c r="B8" s="65" t="s">
+        <v>64</v>
+      </c>
       <c r="C8" s="71"/>
-      <c r="D8" s="109"/>
+      <c r="D8" s="109">
+        <v>480</v>
+      </c>
       <c r="E8" s="108">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="74"/>
-      <c r="B9" s="71"/>
-      <c r="C9" s="71"/>
-      <c r="D9" s="109"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="27">
+      <c r="A9" s="74">
+        <v>2</v>
+      </c>
+      <c r="B9" s="71" t="s">
+        <v>65</v>
+      </c>
+      <c r="C9" s="71" t="s">
+        <v>66</v>
+      </c>
+      <c r="D9" s="109">
+        <v>450</v>
+      </c>
       <c r="E9" s="108">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="71"/>
-      <c r="B10" s="79"/>
+    <row r="10" spans="1:6" ht="27">
+      <c r="A10" s="71">
+        <v>3</v>
+      </c>
+      <c r="B10" s="79" t="s">
+        <v>67</v>
+      </c>
       <c r="C10" s="95"/>
-      <c r="D10" s="113"/>
+      <c r="D10" s="113">
+        <v>240</v>
+      </c>
       <c r="E10" s="108">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="67"/>
-      <c r="B11" s="65"/>
+    <row r="11" spans="1:6" ht="27">
+      <c r="A11" s="67">
+        <v>4</v>
+      </c>
+      <c r="B11" s="65" t="s">
+        <v>68</v>
+      </c>
       <c r="C11" s="98"/>
-      <c r="D11" s="114"/>
+      <c r="D11" s="114">
+        <v>210</v>
+      </c>
       <c r="E11" s="115">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="74"/>
-      <c r="B12" s="71"/>
-      <c r="C12" s="71"/>
-      <c r="D12" s="72"/>
-      <c r="E12" s="74"/>
+    <row r="12" spans="1:6" ht="27">
+      <c r="A12" s="74">
+        <v>5</v>
+      </c>
+      <c r="B12" s="71" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="71" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="72">
+        <v>200</v>
+      </c>
+      <c r="E12" s="74">
+        <v>1</v>
+      </c>
       <c r="F12"/>
     </row>
-    <row r="13" spans="1:6">
-      <c r="A13" s="67"/>
-      <c r="B13" s="65"/>
-      <c r="C13" s="64"/>
-      <c r="D13" s="65"/>
-      <c r="E13" s="74"/>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="67"/>
-      <c r="B14" s="77"/>
-      <c r="C14" s="78"/>
-      <c r="D14" s="77"/>
-      <c r="E14" s="79"/>
+    <row r="13" spans="1:6" ht="27">
+      <c r="A13" s="67">
+        <v>6</v>
+      </c>
+      <c r="B13" s="65" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" s="64" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" s="65">
+        <v>200</v>
+      </c>
+      <c r="E13" s="74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="27">
+      <c r="A14" s="67">
+        <v>7</v>
+      </c>
+      <c r="B14" s="77" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" s="78" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" s="77">
+        <v>170</v>
+      </c>
+      <c r="E14" s="79">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="67"/>
-      <c r="B15" s="65"/>
-      <c r="C15" s="65"/>
-      <c r="D15" s="65"/>
-      <c r="E15" s="74"/>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" s="67"/>
-      <c r="B16" s="65"/>
-      <c r="C16" s="65"/>
-      <c r="D16" s="80"/>
-      <c r="E16" s="74"/>
+      <c r="A15" s="67">
+        <v>8</v>
+      </c>
+      <c r="B15" s="65" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" s="65" t="s">
+        <v>76</v>
+      </c>
+      <c r="D15" s="65">
+        <v>60</v>
+      </c>
+      <c r="E15" s="74">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="27">
+      <c r="A16" s="67">
+        <v>9</v>
+      </c>
+      <c r="B16" s="65" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16" s="65" t="s">
+        <v>78</v>
+      </c>
+      <c r="D16" s="80">
+        <v>60</v>
+      </c>
+      <c r="E16" s="74">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="67"/>
-      <c r="B17" s="77"/>
-      <c r="C17" s="77"/>
-      <c r="D17" s="80"/>
-      <c r="E17" s="67"/>
+      <c r="A17" s="67">
+        <v>10</v>
+      </c>
+      <c r="B17" s="77" t="s">
+        <v>79</v>
+      </c>
+      <c r="C17" s="77" t="s">
+        <v>80</v>
+      </c>
+      <c r="D17" s="80">
+        <v>40</v>
+      </c>
+      <c r="E17" s="67">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="67"/>
@@ -43197,8 +44643,8 @@
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
       <c r="D20" s="7">
-        <f>SUM(D8:D19)</f>
-        <v>0</v>
+        <f>SUM(D8:D17)</f>
+        <v>2110</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.75" thickTop="1">
@@ -43262,22 +44708,38 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="15.75" thickTop="1">
-      <c r="A8" s="76"/>
-      <c r="B8" s="71"/>
-      <c r="C8" s="93"/>
-      <c r="D8" s="109"/>
+    <row r="8" spans="1:7" ht="27.75" thickTop="1">
+      <c r="A8" s="76">
+        <v>1</v>
+      </c>
+      <c r="B8" s="71" t="s">
+        <v>81</v>
+      </c>
+      <c r="C8" s="93" t="s">
+        <v>82</v>
+      </c>
+      <c r="D8" s="109">
+        <v>200</v>
+      </c>
       <c r="E8" s="105">
         <v>1</v>
       </c>
       <c r="F8" s="37"/>
       <c r="G8" s="36"/>
     </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="76"/>
-      <c r="B9" s="71"/>
-      <c r="C9" s="93"/>
-      <c r="D9" s="109"/>
+    <row r="9" spans="1:7" ht="27">
+      <c r="A9" s="76">
+        <v>2</v>
+      </c>
+      <c r="B9" s="71" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="93" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" s="109">
+        <v>120</v>
+      </c>
       <c r="E9" s="105">
         <v>1</v>
       </c>
@@ -43285,10 +44747,18 @@
       <c r="G9" s="36"/>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="76"/>
-      <c r="B10" s="71"/>
-      <c r="C10" s="71"/>
-      <c r="D10" s="109"/>
+      <c r="A10" s="76">
+        <v>3</v>
+      </c>
+      <c r="B10" s="71" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="71" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" s="109">
+        <v>70</v>
+      </c>
       <c r="E10" s="105">
         <v>1</v>
       </c>
@@ -43296,10 +44766,18 @@
       <c r="G10" s="36"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="76"/>
-      <c r="B11" s="71"/>
-      <c r="C11" s="71"/>
-      <c r="D11" s="109"/>
+      <c r="A11" s="76">
+        <v>4</v>
+      </c>
+      <c r="B11" s="71" t="s">
+        <v>87</v>
+      </c>
+      <c r="C11" s="71" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11" s="109">
+        <v>50</v>
+      </c>
       <c r="E11" s="105">
         <v>1</v>
       </c>
@@ -43307,20 +44785,38 @@
       <c r="G11" s="36"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="76"/>
-      <c r="B12" s="71"/>
-      <c r="C12" s="71"/>
-      <c r="D12" s="109"/>
-      <c r="E12" s="62"/>
+      <c r="A12" s="76">
+        <v>5</v>
+      </c>
+      <c r="B12" s="71" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" s="71" t="s">
+        <v>90</v>
+      </c>
+      <c r="D12" s="109">
+        <v>30</v>
+      </c>
+      <c r="E12" s="62">
+        <v>1</v>
+      </c>
       <c r="F12" s="37"/>
       <c r="G12" s="36"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="76"/>
-      <c r="B13" s="71"/>
+      <c r="A13" s="76">
+        <v>6</v>
+      </c>
+      <c r="B13" s="71" t="s">
+        <v>91</v>
+      </c>
       <c r="C13" s="71"/>
-      <c r="D13" s="109"/>
-      <c r="E13" s="62"/>
+      <c r="D13" s="109">
+        <v>10</v>
+      </c>
+      <c r="E13" s="62">
+        <v>1</v>
+      </c>
       <c r="F13" s="37"/>
       <c r="G13" s="36"/>
     </row>
@@ -43386,8 +44882,8 @@
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
       <c r="D22" s="7">
-        <f>SUM(D8:D20)</f>
-        <v>0</v>
+        <f>SUM(D8:D13)</f>
+        <v>480</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="15.75" thickTop="1"/>
@@ -43450,56 +44946,100 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="15.75" thickTop="1">
-      <c r="A8" s="61"/>
-      <c r="B8" s="96"/>
-      <c r="C8" s="96"/>
-      <c r="D8" s="110"/>
+    <row r="8" spans="1:5" ht="30.75" thickTop="1">
+      <c r="A8" s="61">
+        <v>1</v>
+      </c>
+      <c r="B8" s="96" t="s">
+        <v>92</v>
+      </c>
+      <c r="C8" s="96" t="s">
+        <v>93</v>
+      </c>
+      <c r="D8" s="110">
+        <v>780</v>
+      </c>
       <c r="E8" s="119">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="61"/>
-      <c r="B9" s="71"/>
+      <c r="A9" s="61">
+        <v>2</v>
+      </c>
+      <c r="B9" s="71" t="s">
+        <v>94</v>
+      </c>
       <c r="C9" s="71"/>
-      <c r="D9" s="109"/>
+      <c r="D9" s="109">
+        <v>300</v>
+      </c>
       <c r="E9" s="119">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="70"/>
-      <c r="B10" s="71"/>
-      <c r="C10" s="71"/>
-      <c r="D10" s="109"/>
+    <row r="10" spans="1:5" ht="40.5">
+      <c r="A10" s="70">
+        <v>3</v>
+      </c>
+      <c r="B10" s="71" t="s">
+        <v>95</v>
+      </c>
+      <c r="C10" s="71" t="s">
+        <v>96</v>
+      </c>
+      <c r="D10" s="109">
+        <v>195</v>
+      </c>
       <c r="E10" s="120">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="90"/>
-      <c r="B11" s="71"/>
-      <c r="C11" s="93"/>
-      <c r="D11" s="109"/>
+      <c r="A11" s="90">
+        <v>4</v>
+      </c>
+      <c r="B11" s="71" t="s">
+        <v>97</v>
+      </c>
+      <c r="C11" s="93" t="s">
+        <v>98</v>
+      </c>
+      <c r="D11" s="109">
+        <v>170</v>
+      </c>
       <c r="E11" s="120">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
-      <c r="A12" s="90"/>
-      <c r="B12" s="71"/>
-      <c r="C12" s="93"/>
-      <c r="D12" s="109"/>
+    <row r="12" spans="1:5" ht="27">
+      <c r="A12" s="90">
+        <v>5</v>
+      </c>
+      <c r="B12" s="71" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="93" t="s">
+        <v>100</v>
+      </c>
+      <c r="D12" s="109">
+        <v>90</v>
+      </c>
       <c r="E12" s="120">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="70"/>
-      <c r="B13" s="96"/>
+      <c r="A13" s="70">
+        <v>6</v>
+      </c>
+      <c r="B13" s="96" t="s">
+        <v>101</v>
+      </c>
       <c r="C13" s="96"/>
-      <c r="D13" s="110"/>
+      <c r="D13" s="110">
+        <v>30</v>
+      </c>
       <c r="E13" s="120">
         <v>1</v>
       </c>
@@ -43551,8 +45091,8 @@
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
       <c r="D21" s="7">
-        <f>SUM(D8:D20)</f>
-        <v>0</v>
+        <f>SUM(D8:D13)</f>
+        <v>1565</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15.75" thickTop="1"/>

</xml_diff>